<commit_message>
H18: la zona manual recibe veredicto y avisos; --exigir-roi la frena
</commit_message>
<xml_diff>
--- a/data/processed_data/Video_613/contracciones_Video_613.xlsx
+++ b/data/processed_data/Video_613/contracciones_Video_613.xlsx
@@ -779,7 +779,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BM2"/>
+  <dimension ref="A1:BN2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -945,165 +945,170 @@
       </c>
       <c r="AG1" t="inlineStr">
         <is>
+          <t>amplitud_px</t>
+        </is>
+      </c>
+      <c r="AH1" t="inlineStr">
+        <is>
           <t>ttp_n_eventos</t>
         </is>
       </c>
-      <c r="AH1" t="inlineStr">
+      <c r="AI1" t="inlineStr">
         <is>
           <t>ttp_n_medibles</t>
         </is>
       </c>
-      <c r="AI1" t="inlineStr">
+      <c r="AJ1" t="inlineStr">
         <is>
           <t>ttp_frames_mediana</t>
         </is>
       </c>
-      <c r="AJ1" t="inlineStr">
+      <c r="AK1" t="inlineStr">
         <is>
           <t>ttp_reportable</t>
         </is>
       </c>
-      <c r="AK1" t="inlineStr">
+      <c r="AL1" t="inlineStr">
         <is>
           <t>ttp_s</t>
         </is>
       </c>
-      <c r="AL1" t="inlineStr">
+      <c r="AM1" t="inlineStr">
         <is>
           <t>ttp_iqr_s</t>
         </is>
       </c>
-      <c r="AM1" t="inlineStr">
+      <c r="AN1" t="inlineStr">
         <is>
           <t>ttp_cota_inf_s</t>
         </is>
       </c>
-      <c r="AN1" t="inlineStr">
+      <c r="AO1" t="inlineStr">
         <is>
           <t>ttp_cota_sup_s</t>
         </is>
       </c>
-      <c r="AO1" t="inlineStr">
+      <c r="AP1" t="inlineStr">
         <is>
           <t>rt50_n_eventos</t>
         </is>
       </c>
-      <c r="AP1" t="inlineStr">
+      <c r="AQ1" t="inlineStr">
         <is>
           <t>rt50_n_medibles</t>
         </is>
       </c>
-      <c r="AQ1" t="inlineStr">
+      <c r="AR1" t="inlineStr">
         <is>
           <t>rt50_frames_mediana</t>
         </is>
       </c>
-      <c r="AR1" t="inlineStr">
+      <c r="AS1" t="inlineStr">
         <is>
           <t>rt50_reportable</t>
         </is>
       </c>
-      <c r="AS1" t="inlineStr">
+      <c r="AT1" t="inlineStr">
         <is>
           <t>rt50_s</t>
         </is>
       </c>
-      <c r="AT1" t="inlineStr">
+      <c r="AU1" t="inlineStr">
         <is>
           <t>rt50_iqr_s</t>
         </is>
       </c>
-      <c r="AU1" t="inlineStr">
+      <c r="AV1" t="inlineStr">
         <is>
           <t>rt50_cota_inf_s</t>
         </is>
       </c>
-      <c r="AV1" t="inlineStr">
+      <c r="AW1" t="inlineStr">
         <is>
           <t>rt50_cota_sup_s</t>
         </is>
       </c>
-      <c r="AW1" t="inlineStr">
+      <c r="AX1" t="inlineStr">
         <is>
           <t>cinetica_motivo</t>
         </is>
       </c>
-      <c r="AX1" t="inlineStr">
+      <c r="AY1" t="inlineStr">
         <is>
           <t>fotogramas_sin_medida</t>
         </is>
       </c>
-      <c r="AY1" t="inlineStr">
+      <c r="AZ1" t="inlineStr">
         <is>
           <t>fotogramas_sin_medida_pct</t>
         </is>
       </c>
-      <c r="AZ1" t="inlineStr">
+      <c r="BA1" t="inlineStr">
         <is>
           <t>fotogramas_low_quality</t>
         </is>
       </c>
-      <c r="BA1" t="inlineStr">
+      <c r="BB1" t="inlineStr">
         <is>
           <t>eventos_junto_a_hueco</t>
         </is>
       </c>
-      <c r="BB1" t="inlineStr">
+      <c r="BC1" t="inlineStr">
         <is>
           <t>eventos_junto_al_borde</t>
         </is>
       </c>
-      <c r="BC1" t="inlineStr">
+      <c r="BD1" t="inlineStr">
         <is>
           <t>win_s_usado</t>
         </is>
       </c>
-      <c r="BD1" t="inlineStr">
+      <c r="BE1" t="inlineStr">
         <is>
           <t>win_s_automatico</t>
         </is>
       </c>
-      <c r="BE1" t="inlineStr">
+      <c r="BF1" t="inlineStr">
         <is>
           <t>duracion_evento_max_s</t>
         </is>
       </c>
-      <c r="BF1" t="inlineStr">
+      <c r="BG1" t="inlineStr">
         <is>
           <t>ventana_corta</t>
         </is>
       </c>
-      <c r="BG1" t="inlineStr">
+      <c r="BH1" t="inlineStr">
         <is>
           <t>conteo_por_ventana</t>
         </is>
       </c>
-      <c r="BH1" t="inlineStr">
+      <c r="BI1" t="inlineStr">
         <is>
           <t>conteo_estable_ventana</t>
         </is>
       </c>
-      <c r="BI1" t="inlineStr">
+      <c r="BJ1" t="inlineStr">
         <is>
           <t>mesetas</t>
         </is>
       </c>
-      <c r="BJ1" t="inlineStr">
+      <c r="BK1" t="inlineStr">
         <is>
           <t>motivo_no_reportable</t>
         </is>
       </c>
-      <c r="BK1" t="inlineStr">
+      <c r="BL1" t="inlineStr">
         <is>
           <t>ruido_borde_sup_px</t>
         </is>
       </c>
-      <c r="BL1" t="inlineStr">
+      <c r="BM1" t="inlineStr">
         <is>
           <t>ruido_borde_inf_px</t>
         </is>
       </c>
-      <c r="BM1" t="inlineStr">
+      <c r="BN1" t="inlineStr">
         <is>
           <t>cociente_ruido_bordes</t>
         </is>
@@ -1260,53 +1265,53 @@
         </is>
       </c>
       <c r="AG2" t="n">
+        <v>0.3198999999999614</v>
+      </c>
+      <c r="AH2" t="n">
         <v>24</v>
       </c>
-      <c r="AH2" t="n">
-        <v>0</v>
-      </c>
       <c r="AI2" t="n">
-        <v>1</v>
-      </c>
-      <c r="AJ2" t="b">
-        <v>0</v>
-      </c>
-      <c r="AK2" t="inlineStr"/>
+        <v>0</v>
+      </c>
+      <c r="AJ2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AK2" t="b">
+        <v>0</v>
+      </c>
       <c r="AL2" t="inlineStr"/>
-      <c r="AM2" t="n">
-        <v>0</v>
-      </c>
+      <c r="AM2" t="inlineStr"/>
       <c r="AN2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AO2" t="n">
         <v>0.08083333333333131</v>
       </c>
-      <c r="AO2" t="n">
+      <c r="AP2" t="n">
         <v>24</v>
       </c>
-      <c r="AP2" t="n">
-        <v>0</v>
-      </c>
       <c r="AQ2" t="n">
-        <v>1</v>
-      </c>
-      <c r="AR2" t="b">
-        <v>0</v>
-      </c>
-      <c r="AS2" t="inlineStr"/>
+        <v>0</v>
+      </c>
+      <c r="AR2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AS2" t="b">
+        <v>0</v>
+      </c>
       <c r="AT2" t="inlineStr"/>
-      <c r="AU2" t="n">
-        <v>0</v>
-      </c>
+      <c r="AU2" t="inlineStr"/>
       <c r="AV2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AW2" t="n">
         <v>0.06750000000000256</v>
       </c>
-      <c r="AW2" t="inlineStr">
+      <c r="AX2" t="inlineStr">
         <is>
           <t>TTP: el conteo de eventos no es reportable; RT50: el conteo de eventos no es reportable</t>
         </is>
       </c>
-      <c r="AX2" t="n">
-        <v>0</v>
-      </c>
       <c r="AY2" t="n">
         <v>0</v>
       </c>
@@ -1317,41 +1322,44 @@
         <v>0</v>
       </c>
       <c r="BB2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="BC2" t="n">
+        <v>1</v>
+      </c>
+      <c r="BD2" t="n">
         <v>2</v>
       </c>
-      <c r="BD2" t="b">
-        <v>1</v>
-      </c>
-      <c r="BE2" t="n">
+      <c r="BE2" t="b">
+        <v>1</v>
+      </c>
+      <c r="BF2" t="n">
         <v>0.09999999999999432</v>
       </c>
-      <c r="BF2" t="b">
-        <v>0</v>
-      </c>
-      <c r="BG2" t="inlineStr">
+      <c r="BG2" t="b">
+        <v>0</v>
+      </c>
+      <c r="BH2" t="inlineStr">
         <is>
           <t>1.5 s: sin meseta | 2 s: sin meseta | 3 s: sin meseta</t>
         </is>
       </c>
-      <c r="BH2" t="b">
-        <v>0</v>
-      </c>
-      <c r="BI2" t="inlineStr"/>
-      <c r="BJ2" t="inlineStr">
+      <c r="BI2" t="b">
+        <v>0</v>
+      </c>
+      <c r="BJ2" t="inlineStr"/>
+      <c r="BK2" t="inlineStr">
         <is>
           <t>no hay meseta en el escaneo de k</t>
         </is>
       </c>
-      <c r="BK2" t="n">
+      <c r="BL2" t="n">
         <v>0.03617544000002103</v>
       </c>
-      <c r="BL2" t="n">
+      <c r="BM2" t="n">
         <v>0.04166105999999244</v>
       </c>
-      <c r="BM2" t="n">
+      <c r="BN2" t="n">
         <v>1.151639344261417</v>
       </c>
     </row>
@@ -4400,7 +4408,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V3"/>
+  <dimension ref="A1:W3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4431,85 +4439,90 @@
       </c>
       <c r="F1" t="inlineStr">
         <is>
+          <t>amplitud_px</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
           <t>ttp_n_eventos</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>ttp_n_medibles</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>ttp_frames_mediana</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>ttp_reportable</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>ttp_s</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>ttp_iqr_s</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>ttp_cota_inf_s</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="N1" t="inlineStr">
         <is>
           <t>ttp_cota_sup_s</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="O1" t="inlineStr">
         <is>
           <t>rt50_n_eventos</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr">
+      <c r="P1" t="inlineStr">
         <is>
           <t>rt50_n_medibles</t>
         </is>
       </c>
-      <c r="P1" t="inlineStr">
+      <c r="Q1" t="inlineStr">
         <is>
           <t>rt50_frames_mediana</t>
         </is>
       </c>
-      <c r="Q1" t="inlineStr">
+      <c r="R1" t="inlineStr">
         <is>
           <t>rt50_reportable</t>
         </is>
       </c>
-      <c r="R1" t="inlineStr">
+      <c r="S1" t="inlineStr">
         <is>
           <t>rt50_s</t>
         </is>
       </c>
-      <c r="S1" t="inlineStr">
+      <c r="T1" t="inlineStr">
         <is>
           <t>rt50_iqr_s</t>
         </is>
       </c>
-      <c r="T1" t="inlineStr">
+      <c r="U1" t="inlineStr">
         <is>
           <t>rt50_cota_inf_s</t>
         </is>
       </c>
-      <c r="U1" t="inlineStr">
+      <c r="V1" t="inlineStr">
         <is>
           <t>rt50_cota_sup_s</t>
         </is>
       </c>
-      <c r="V1" t="inlineStr">
+      <c r="W1" t="inlineStr">
         <is>
           <t>cinetica_motivo</t>
         </is>
@@ -4536,46 +4549,49 @@
         </is>
       </c>
       <c r="F2" t="n">
+        <v>0.3198999999999614</v>
+      </c>
+      <c r="G2" t="n">
         <v>24</v>
       </c>
-      <c r="G2" t="n">
-        <v>0</v>
-      </c>
       <c r="H2" t="n">
-        <v>1</v>
-      </c>
-      <c r="I2" t="b">
-        <v>0</v>
-      </c>
-      <c r="J2" t="inlineStr"/>
+        <v>0</v>
+      </c>
+      <c r="I2" t="n">
+        <v>1</v>
+      </c>
+      <c r="J2" t="b">
+        <v>0</v>
+      </c>
       <c r="K2" t="inlineStr"/>
-      <c r="L2" t="n">
-        <v>0</v>
-      </c>
+      <c r="L2" t="inlineStr"/>
       <c r="M2" t="n">
+        <v>0</v>
+      </c>
+      <c r="N2" t="n">
         <v>0.08083333333333131</v>
       </c>
-      <c r="N2" t="n">
+      <c r="O2" t="n">
         <v>24</v>
       </c>
-      <c r="O2" t="n">
-        <v>0</v>
-      </c>
       <c r="P2" t="n">
-        <v>1</v>
-      </c>
-      <c r="Q2" t="b">
-        <v>0</v>
-      </c>
-      <c r="R2" t="inlineStr"/>
+        <v>0</v>
+      </c>
+      <c r="Q2" t="n">
+        <v>1</v>
+      </c>
+      <c r="R2" t="b">
+        <v>0</v>
+      </c>
       <c r="S2" t="inlineStr"/>
-      <c r="T2" t="n">
-        <v>0</v>
-      </c>
+      <c r="T2" t="inlineStr"/>
       <c r="U2" t="n">
+        <v>0</v>
+      </c>
+      <c r="V2" t="n">
         <v>0.06750000000000256</v>
       </c>
-      <c r="V2" t="inlineStr">
+      <c r="W2" t="inlineStr">
         <is>
           <t>TTP: el conteo de eventos no es reportable; RT50: el conteo de eventos no es reportable</t>
         </is>
@@ -4602,46 +4618,49 @@
         </is>
       </c>
       <c r="F3" t="n">
+        <v>0.3198999999999614</v>
+      </c>
+      <c r="G3" t="n">
         <v>24</v>
       </c>
-      <c r="G3" t="n">
-        <v>0</v>
-      </c>
       <c r="H3" t="n">
-        <v>1</v>
-      </c>
-      <c r="I3" t="b">
-        <v>0</v>
-      </c>
-      <c r="J3" t="inlineStr"/>
+        <v>0</v>
+      </c>
+      <c r="I3" t="n">
+        <v>1</v>
+      </c>
+      <c r="J3" t="b">
+        <v>0</v>
+      </c>
       <c r="K3" t="inlineStr"/>
-      <c r="L3" t="n">
-        <v>0</v>
-      </c>
+      <c r="L3" t="inlineStr"/>
       <c r="M3" t="n">
+        <v>0</v>
+      </c>
+      <c r="N3" t="n">
         <v>0.08083333333333131</v>
       </c>
-      <c r="N3" t="n">
+      <c r="O3" t="n">
         <v>24</v>
       </c>
-      <c r="O3" t="n">
-        <v>0</v>
-      </c>
       <c r="P3" t="n">
-        <v>1</v>
-      </c>
-      <c r="Q3" t="b">
-        <v>0</v>
-      </c>
-      <c r="R3" t="inlineStr"/>
+        <v>0</v>
+      </c>
+      <c r="Q3" t="n">
+        <v>1</v>
+      </c>
+      <c r="R3" t="b">
+        <v>0</v>
+      </c>
       <c r="S3" t="inlineStr"/>
-      <c r="T3" t="n">
-        <v>0</v>
-      </c>
+      <c r="T3" t="inlineStr"/>
       <c r="U3" t="n">
+        <v>0</v>
+      </c>
+      <c r="V3" t="n">
         <v>0.06750000000000256</v>
       </c>
-      <c r="V3" t="inlineStr">
+      <c r="W3" t="inlineStr">
         <is>
           <t>TTP: el conteo de eventos no es reportable; RT50: el conteo de eventos no es reportable</t>
         </is>

</xml_diff>